<commit_message>
Remove older spells that are not part of these raids.
Drop the listed IDs from the site, spreadsheet, and Word writeup, and keep Sneeze as a mechanic without spell data.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -20,17 +20,17 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Siren Sisters'!$A$1:$G$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Siren Sisters'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dipuc'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dipuc'!$A$1:$G$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$G$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$G$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$G$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$G$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$G$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$G$61</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$G$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
@@ -752,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -801,181 +801,126 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Piercing Shot</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>5720</v>
+        <v>75153</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 250
-Decrease Armor Class by 7 to 9, Based on Class</t>
+          <t>Decrease Current Hit Points by 1600600</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>An arrow slices through your armor.</t>
+          <t>A powerful arrow punches through you.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Piercing Shot</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>39655</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 5000</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Shatter Shot</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>75154</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 800800</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>You are pierced by an arrow.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>A rain of arrows pierce your flesh.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Piercing Shot</t>
+          <t>Scornful Touch</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>75153</v>
+        <v>75156</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 1600600</t>
+          <t>Increase Melee Haste by 10%
+Increase Hit Damage by 10% (v185)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>A powerful arrow punches through you.</t>
-        </is>
-      </c>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="16" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Shatter Shot</t>
+          <t>Curse of the Broken Heart</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>75154</v>
+        <v>75157</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 800800</t>
+          <t>Decrease Current Hit Points by 500500 per Tick
+Decrease Movement Speed by 25%</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>5 ticks</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>A rain of arrows pierce your flesh.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="32" customHeight="1">
+          <t>A painful weight settles in on your chest.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>The weight lifts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Scornful Touch</t>
+          <t>Unrequited Love</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>75156</v>
+        <v>75158</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Increase Melee Haste by 10%
-Increase Hit Damage by 10% (v185)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Curse of the Broken Heart</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>75157</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 500500 per Tick
-Decrease Movement Speed by 25%</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>A painful weight settles in on your chest.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>The weight lifts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="64" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Unrequited Love</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>75158</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 500500
 Decrease Current Hit Points by 750000 per Tick
@@ -983,29 +928,27 @@
 Increase Cast Time by 1s</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>You are filled with deep sadness.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -1026,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1075,21 +1018,18 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="128" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Rapid Fire</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>32119</v>
+        <v>75178</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 62012 (Random: -52500 to -71525)
-Decrease Current Hit Points by 62012 (Random: -52500 to -71525)
-Decrease Current Hit Points by 62012 (Random: -52500 to -71525)
-Decrease Current Hit Points by 62012 (Random: -52500 to -71525)</t>
+          <t>Decrease Current Hit Points by 660000</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -1098,348 +1038,352 @@
           <t>Instant</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>A barbed arrow pierces you.</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Rapid Fire</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>75178</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 660000</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>A barbed arrow pierces you.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Invigorating Essence</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B3" s="5" t="n">
         <v>75184</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Increase Current Mana by 0.25% of Total Mana per Tick, Max: 0
 Increase Current Endurance by 0.25% of Total Endurance per Tick, Max: 0</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>You draw energy from the surrounding area.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>You no longer feel empowered.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Quickened Reflexes</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B4" s="3" t="n">
         <v>75185</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Increase Melee Haste by 45%
 Decrease Cast Time by 0.75s</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Your attacks seem faster.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Your attacks return to normal.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Protective Embrace</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B5" s="5" t="n">
         <v>75182</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Absorb Spell Damage: 15%, Max per Hit: 300000
 Absorb Melee Damage: 15%, Max per Hit: 300000
 Absorb DoT Damage: 15%, Max per Hit: 300000</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>A protective barrier covers you.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>The protective barrier fades.</t>
         </is>
       </c>
     </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Gift of Giving</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>75183</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Increase Healing by 20% (v125, Before Crit)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>A soothing energy fills you.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>The soothing energy fades.</t>
+        </is>
+      </c>
+    </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Gift of Giving</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>75183</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Increase Healing by 20% (v125, Before Crit)</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Briar Shackles</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>75189</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Movement Speed by 250%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>A soothing energy fills you.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>The soothing energy fades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Briar Shackles</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>75189</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Movement Speed by 250%</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Thorned shackles wrap around your legs.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>The shackles shrivel and break.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Draining Touch</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B8" s="3" t="n">
         <v>75186</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Decrease Spell Damage by 1% to 20% (v124, Before DoT Crit, After DD Crit)
 Decrease Hit Damage by 20% (v185)</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Your attacks and spells feel weaker.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>You feel invigorated again.</t>
         </is>
       </c>
     </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sapping Buds</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>75187</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Healing by 1% to 10% (v125, Before Crit)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Flowering buds spring from your skin.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>The flowers bloom and fall away.</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Sapping Buds</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n">
-        <v>75187</v>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Healing by 1% to 10% (v125, Before Crit)</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Languorous Runes</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>75188</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Spell Mana Cost by 25%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Flowering buds spring from your skin.</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>The flowers bloom and fall away.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Languorous Runes</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>75188</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Spell Mana Cost by 25%</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Sapping runes cover your body.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>The runes disappear.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Bramble Shield</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B11" s="5" t="n">
         <v>75192</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 1250
 Increase Chance to Reflect Spell by 15% for 45% Base Damage</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>The barbs fall away.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Coerced Loyalty</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>75200</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Charm up to Level 300
 Decrease Chance of Charm Breaking by 50%</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Your body moves on its own.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>You regain control of your body.</t>
         </is>
       </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Stolen Words</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>75190</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Inhibit Spell Casting (Spell Silence)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>1 tick</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>You find it impossible to form words.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1448,11 +1392,11 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>75190</v>
+        <v>75201</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Inhibit Spell Casting (Spell Silence)</t>
+          <t>Decrease Current Hit Points by 100 per Tick</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr"/>
@@ -1461,46 +1405,19 @@
           <t>1 tick</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>You find it impossible to form words.</t>
-        </is>
-      </c>
+      <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="4" t="inlineStr"/>
     </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Stolen Words</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>75201</v>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 100 per Tick</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>1 tick</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Lucky in Life</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B15" s="3" t="n">
         <v>75195</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Increase Spell Damage by 5% (v124, Before DoT Crit, After DD Crit)
 Increase Hit Damage by 5% (v185)
@@ -1508,58 +1425,58 @@
 Increase Current Endurance by 0.5% of Total Endurance per Tick, Max: 0</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Your inner fire grows to an inferno.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Your inner fire dims.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Unlucky in Life</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B16" s="5" t="n">
         <v>75197</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Decrease Spell Damage by 1% to 10% (v124, Before DoT Crit, After DD Crit)
 Decrease Hit Damage by 10% (v185)
 Stun for 6s</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Your spirit is crushed.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>You refocus on the fight.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17"/>
+  <autoFilter ref="A1:G16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1576,7 +1493,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -1597,7 +1513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1682,31 +1598,30 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>8782</v>
+        <v>52393</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Hand to Hand Attack for 65 with 10000% Accuracy Mod
-Hand to Hand Attack for 65 with 10000% Accuracy Mod
-Hand to Hand Attack for 65 with 10000% Accuracy Mod</t>
+          <t>Decrease Current Hit Points by 135165 per Tick
+Decrease Current Hit Points by 111111</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>3 ticks</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>A shock wave shivers through your body.</t>
+          <t>The griffin rakes with its back claws.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
@@ -1718,23 +1633,23 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>45478</v>
+        <v>75134</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 99999
-Decrease Movement Speed by 35%</t>
+          <t>Decrease Current Hit Points by 600600
+Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>5 ticks</t>
+          <t>2 ticks</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>The cat rakes you across the legs.</t>
+          <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
@@ -1746,290 +1661,207 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>52393</v>
+        <v>75135</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 135165 per Tick
-Decrease Current Hit Points by 111111</t>
+          <t>Decrease Current Hit Points by 600600
+Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>3 ticks</t>
+          <t>2 ticks</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>The griffin rakes with its back claws.</t>
+          <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>75134</v>
+        <v>75151</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 600600
-Inhibit Spell Casting (Spell Silence)</t>
+          <t>Fling</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>2 ticks</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>The manticore's claws rake across your flesh.</t>
+          <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>75135</v>
+        <v>75152</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 600600
-Inhibit Spell Casting (Spell Silence)</t>
+          <t>Fling</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>2 ticks</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>The manticore's claws rake across your flesh.</t>
+          <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
     </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Rake</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>75151</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Fling</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>The manticore's claws strike throws you back.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Rake</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>75152</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Fling</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>The manticore's claws strike throws you back.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Sneeze</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>39118</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Push Back 2 Units and Up 2 Units</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>You are thrown backwards.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Lockjaw Trap</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B8" s="3" t="n">
         <v>75137</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Root</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>The razor sharp jaws of the trap cut into your leg.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Your wounds close.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Slow Your Roll</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>75138</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 750000
 Decrease Melee Haste by 10% (v371, Incremental)
 Increase Cast Time by 1s</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Moruuk's blow rattles you, slowing your reactions.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>You shake off the attack.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Stronger Together</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B10" s="3" t="n">
         <v>75141</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Increase Melee Haste by 25%</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Taking Your Stuff</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B11" s="5" t="n">
         <v>75140</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Mana by 0.1% of Total Mana, Max: 0
 Decrease Current Endurance by 0.1% of Total Endurance, Max: 0</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>You feel drained.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="80" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Aura of Greed</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B12" s="3" t="n">
         <v>75147</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2037,29 +1869,29 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>The weight of your poverty takes its toll.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="80" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Aura of Poverty</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B13" s="5" t="n">
         <v>75148</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2067,21 +1899,21 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>The weight of your greed takes its toll.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2095,9 +1927,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -2393,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2748,81 +2577,44 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Wither</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>39657</v>
+        <v>75113</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Increase Hit Damage Taken by 25%
-Decrease Current Hit Points by 6000 per Tick
-Increase Poison Counter by 10</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Poison 10</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Poison withers your body, you become weak and vulnerable</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>You regain your strength</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Wither</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>75113</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000 per Tick
 Increase Corruption Counter by 30</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Corruption 30</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Corruption drains your life essence.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>The corruption dissipates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2835,7 +2627,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -2856,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3196,82 +2987,82 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7231</v>
+        <v>13023</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Feign Death (1% Chance)
+Decrease Current Hit Points by 50000</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Sharpened horns gore your flesh.</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Minotaur Gore</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>75013</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Feign Death (1% Chance)
+Decrease Current Hit Points by 650000</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Sharpened horns gore your flesh.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Decapitating Chop</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>7234</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 100000</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Sharpened horns gore your flesh.</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Minotaur Gore</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>13023</v>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 50000</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Sharpened horns gore your flesh.</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Minotaur Gore</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>75013</v>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 650000</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Sharpened horns gore your flesh.</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>You are slain by a mighty cleave.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -3280,12 +3071,12 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>7234</v>
+        <v>75014</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 100000</t>
+Decrease Current Hit Points by 4000000000</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
@@ -3301,44 +3092,16 @@
       </c>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Decapitating Chop</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
-        <v>75014</v>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 4000000000</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>You are slain by a mighty cleave.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Malaise</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B16" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Decrease Cold Resist by 20
 Decrease Magic Resist by 20
@@ -3346,101 +3109,61 @@
 Decrease Fire Resist by 20</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>14m</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>You feel somewhat vulnerable.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>Your vulnerability fades.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="64" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Spite</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B17" s="3" t="n">
         <v>40778</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 25000 per Tick (Scales, Base Level: 105)
 Decrease Current Mana by 10000 per Tick (Scales, Base Level: 105) (v417)</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>You are filled with a sense of bitter spite.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="96" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="96" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Spirit Cleaver</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
-        <v>4729</v>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Attack by 500
-Decrease Current Hit Points by 1225 per Tick
-Decrease Current Mana by 400 per Tick
-Decrease Current Endurance by 400 per Tick
-Decrease Base Stats by 350
-Increase Poison Counter by 297</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Poison 297</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>3m 36s</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>An invisible force of rage splits your soul in two.</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>You feel whole again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="96" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Spirit Cleaver</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
+      <c r="B18" s="5" t="n">
         <v>75024</v>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Decrease Attack by 500
 Decrease Current Hit Points by 122500 per Tick
@@ -3450,247 +3173,93 @@
 Increase Poison Counter by 297</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Poison 297</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>3m 36s</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>An invisible force of rage splits your soul in two.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>You feel whole again.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Soul Consumption</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
-        <v>852</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 2700
-Decrease Current Mana by 2700</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>An invisible force tugs at your soul.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Soul Consumption</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>1930</v>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 50 per Tick</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>You feel your life force drain away.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>The bond fades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Soul Consumption</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>17141</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 500 per Tick</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>You feel your life force drain away.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>The bond fades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Soul Consumption</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
+      <c r="B19" s="3" t="n">
         <v>75056</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 375000
 Decrease Current Mana by 2700</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Spear of Discord</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
-        <v>4727</v>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 6175
-Stun NPC for 10s (PC for 5.25s)</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Your body is pierced by the spear of discord.</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Spear of Discord</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>75057</v>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 425000
 Stun NPC for 10s (PC for 5.25s)</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27" ht="96" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="96" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Wave of Rage</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
-        <v>4728</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Increase Spell Mana Cost by 1% to 50%
-Decrease Current Hit Points by 4050
-Decrease Current Hit Points by 500 per Tick
-Decrease Intelligence by 400
-Decrease Wisdom by 400
-Increase Poison Counter by 396</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Poison 396</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Your spirit is overcome by a wave of rage.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28" ht="96" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Wave of Rage</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n">
+      <c r="B21" s="3" t="n">
         <v>75023</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Increase Spell Mana Cost by 1% to 50%
 Decrease Current Hit Points by 325000
@@ -3700,72 +3269,248 @@
 Increase Poison Counter by 396</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Poison 396</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Ikaav Venom</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B22" s="5" t="n">
         <v>17057</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 7500
 Decrease Current Hit Points by 5000 per Tick
 Increase Poison Counter by 50</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>Poison 50</t>
         </is>
       </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>10m</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Poison courses through your system after you were bitten.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>You sigh in relief as the poison fades away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Discord's Rebuke</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>75025</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 475000</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Chaos fills your mind and pains your soul.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Vis Percussio</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>48039</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Vis Percussio</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>75033</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>48040</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>75034</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Vita Tardius</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>75031</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 222000 per Tick
+Decrease Melee Haste by 55%</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Your body convulses as electricity runs through you.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Vita Tardius</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>75039</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Melee Haste by 55% (v371, Incremental)
+Decrease Current Hit Points by 150000 per Tick</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>10m</t>
+          <t>5 ticks</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Poison courses through your system after you were bitten.</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>You sigh in relief as the poison fades away.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
+          <t>Your body convulses as electricity runs through you.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Discord's Rebuke</t>
+          <t>Claustro Vitoris</t>
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>4739</v>
+        <v>75030</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 3000</t>
+          <t>Decrease Current Hit Points by 325000
+Stun for 1s</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
@@ -3776,23 +3521,24 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Chaos fills your mind and pains your soul.</t>
+          <t>You are shocked!</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
     </row>
-    <row r="31" ht="16" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Discord's Rebuke</t>
+          <t>Claustro Vitoris</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>75025</v>
+        <v>75035</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 475000</t>
+          <t>Decrease Current Hit Points by 350000
+Stun for 1s</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
@@ -3803,674 +3549,161 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Chaos fills your mind and pains your soul.</t>
+          <t>You are shocked!</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
     </row>
-    <row r="32" ht="16" customHeight="1">
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Vis Percussio</t>
+          <t>Claustro Facultis</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>48039</v>
+        <v>75036</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Decrease Current Hit Points by 275000
+Decrease Current Mana by 3510 (v417)</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Magic drains painfully from your body.</t>
+        </is>
+      </c>
       <c r="G32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Vis Percussio</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>75033</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use:</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>48040</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use:</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>75034</v>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use:</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>47479</v>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 33330 per Tick
-Decrease Melee Haste by 55%</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>48045</v>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Melee Haste by 55% (v371, Incremental)
-Decrease Current Hit Points by 22122 per Tick</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="n">
-        <v>75031</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 222000 per Tick
-Decrease Melee Haste by 55%</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>75039</v>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Melee Haste by 55% (v371, Incremental)
-Decrease Current Hit Points by 150000 per Tick</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>47478</v>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 65000
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="n">
-        <v>48041</v>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 96148
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>75030</v>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="32" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="n">
-        <v>75035</v>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 350000
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44" ht="32" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Claustro Facultis</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>48042</v>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 87880
-Decrease Current Mana by 3510 (v417)</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Magic drains painfully from your body.</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Claustro Facultis</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>75036</v>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 275000
-Decrease Current Mana by 3510 (v417)</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Magic drains painfully from your body.</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Repenta Vitoris</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
-        <v>47480</v>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 37892 per Tick</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="B33" s="3" t="n">
+        <v>75032</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 456789 per Tick</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>A ball of electricity gathers around you.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Repenta Vitoris</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="n">
-        <v>48046</v>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 29147 per Tick</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>A ball of electricity gathers around you.</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Repenta Vitoris</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>75032</v>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 456789 per Tick</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>A ball of electricity gathers around you.</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="32" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>Ignas Maxio</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
-        <v>48043</v>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 45999 per Tick
-Decrease Movement Speed by 65%</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Flames engulf you.</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50" ht="32" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>Ignas Maxio</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n">
+      <c r="B34" s="5" t="n">
         <v>75037</v>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 299000 per Tick
 Decrease Movement Speed by 65%</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Flames engulf you.</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51" ht="48" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Humas Maxio</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
-        <v>48044</v>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 88560
-Push Back 3 Units and Up 3 Units
-Stun for 2s</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>You are engulfed in grinding earth.</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52" ht="48" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Humas Maxio</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="n">
+      <c r="B35" s="3" t="n">
         <v>75038</v>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 444000
 Push Back 3 Units and Up 3 Units
 Stun for 2s</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>You are engulfed in grinding earth.</t>
         </is>
       </c>
-      <c r="G52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Gravitas Maxio</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
-        <v>48047</v>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
-Decrease Current Hit Points by 19543 per Tick</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr"/>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>2 ticks</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>You feel the very earth pulling you apart.</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>Gravitas Maxio</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="n">
+      <c r="B36" s="5" t="n">
         <v>75040</v>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
 Decrease Current Hit Points by 175000 per Tick</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr"/>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>You feel the very earth pulling you apart.</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55" ht="64" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="G36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="64" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>Resonating Beam</t>
         </is>
       </c>
-      <c r="B55" s="3" t="n">
-        <v>48051</v>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Dispel Beneficial (100% Chance)
-Decrease Current Hit Points by 112000
-Decrease Current Mana by 4500 (v417)
-Decrease Current Endurance by 1850</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>You are hit by a powerful resonation.</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56" ht="64" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Resonating Beam</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n">
+      <c r="B37" s="3" t="n">
         <v>75058</v>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Dispel Beneficial (100% Chance)
 Decrease Current Hit Points by 600000
@@ -4478,128 +3711,565 @@
 Decrease Current Endurance by 1850</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>You are hit by a powerful resonation.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="32" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Repulsion of the First Creation</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n">
+      <c r="B38" s="5" t="n">
         <v>23056</v>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 10000
 Push Back 3 Units and Up 12 Units</t>
         </is>
       </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>You are repulsed.</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="32" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Repulsion of the First Creation</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>75042</v>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 125000
+Push Back 3 Units and Up 12 Units</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>You are repulsed.</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Retribution of the First Creation</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>23077</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 12000</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Retribution of the First Creation</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>75053</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 325000</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>23057</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 100</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>23058</v>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 200</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>23059</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 300</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>23060</v>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 400</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>23061</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 500</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>23062</v>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 600</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>23063</v>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 700</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>23064</v>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 800</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>23065</v>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 900</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>23066</v>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 1000</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>75043</v>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 1000</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr"/>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>75044</v>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 2000</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr"/>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>75045</v>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 3000</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr"/>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>75046</v>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 4000</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr"/>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>75047</v>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 5000</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr"/>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>75048</v>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 6000</t>
+        </is>
+      </c>
       <c r="D57" s="4" t="inlineStr"/>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr"/>
       <c r="G57" s="4" t="inlineStr"/>
     </row>
-    <row r="58" ht="32" customHeight="1">
+    <row r="58" ht="16" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>Repulsion of the First Creation</t>
+          <t>Lava Elemental Protection</t>
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>75042</v>
+        <v>75049</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 125000
-Push Back 3 Units and Up 12 Units</t>
+          <t>Increase Damage Shield by 7000</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr"/>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr"/>
       <c r="G58" s="4" t="inlineStr"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="n">
-        <v>23077</v>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 12000</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60" ht="32" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="n">
-        <v>75053</v>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr"/>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>75050</v>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 8000</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr"/>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>75051</v>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 16000</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr"/>
+      <c r="G60" s="4" t="inlineStr"/>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
@@ -4608,11 +4278,11 @@
         </is>
       </c>
       <c r="B61" s="5" t="n">
-        <v>23057</v>
+        <v>75052</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 100</t>
+          <t>Increase Damage Shield by 32000</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr"/>
@@ -4624,445 +4294,8 @@
       <c r="F61" s="4" t="inlineStr"/>
       <c r="G61" s="4" t="inlineStr"/>
     </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B62" s="5" t="n">
-        <v>23058</v>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 200</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr"/>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr"/>
-      <c r="G62" s="4" t="inlineStr"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="n">
-        <v>23059</v>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 300</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr"/>
-      <c r="E63" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F63" s="4" t="inlineStr"/>
-      <c r="G63" s="4" t="inlineStr"/>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B64" s="5" t="n">
-        <v>23060</v>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 400</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr"/>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr"/>
-      <c r="G64" s="4" t="inlineStr"/>
-    </row>
-    <row r="65" ht="16" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B65" s="5" t="n">
-        <v>23061</v>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 500</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr"/>
-      <c r="E65" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F65" s="4" t="inlineStr"/>
-      <c r="G65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="n">
-        <v>23062</v>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 600</t>
-        </is>
-      </c>
-      <c r="D66" s="4" t="inlineStr"/>
-      <c r="E66" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F66" s="4" t="inlineStr"/>
-      <c r="G66" s="4" t="inlineStr"/>
-    </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="n">
-        <v>23063</v>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 700</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr"/>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr"/>
-      <c r="G67" s="4" t="inlineStr"/>
-    </row>
-    <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="n">
-        <v>23064</v>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 800</t>
-        </is>
-      </c>
-      <c r="D68" s="4" t="inlineStr"/>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr"/>
-      <c r="G68" s="4" t="inlineStr"/>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B69" s="5" t="n">
-        <v>23065</v>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 900</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr"/>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr"/>
-      <c r="G69" s="4" t="inlineStr"/>
-    </row>
-    <row r="70" ht="16" customHeight="1">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B70" s="5" t="n">
-        <v>23066</v>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr"/>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr"/>
-      <c r="G70" s="4" t="inlineStr"/>
-    </row>
-    <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B71" s="5" t="n">
-        <v>75043</v>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr"/>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr"/>
-      <c r="G71" s="4" t="inlineStr"/>
-    </row>
-    <row r="72" ht="16" customHeight="1">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="n">
-        <v>75044</v>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 2000</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr"/>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr"/>
-      <c r="G72" s="4" t="inlineStr"/>
-    </row>
-    <row r="73" ht="16" customHeight="1">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B73" s="5" t="n">
-        <v>75045</v>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 3000</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr"/>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="4" t="inlineStr"/>
-    </row>
-    <row r="74" ht="16" customHeight="1">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="n">
-        <v>75046</v>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 4000</t>
-        </is>
-      </c>
-      <c r="D74" s="4" t="inlineStr"/>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr"/>
-      <c r="G74" s="4" t="inlineStr"/>
-    </row>
-    <row r="75" ht="16" customHeight="1">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B75" s="5" t="n">
-        <v>75047</v>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 5000</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr"/>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr"/>
-      <c r="G75" s="4" t="inlineStr"/>
-    </row>
-    <row r="76" ht="16" customHeight="1">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B76" s="5" t="n">
-        <v>75048</v>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 6000</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr"/>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr"/>
-      <c r="G76" s="4" t="inlineStr"/>
-    </row>
-    <row r="77" ht="16" customHeight="1">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B77" s="5" t="n">
-        <v>75049</v>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 7000</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr"/>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr"/>
-      <c r="G77" s="4" t="inlineStr"/>
-    </row>
-    <row r="78" ht="16" customHeight="1">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="n">
-        <v>75050</v>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 8000</t>
-        </is>
-      </c>
-      <c r="D78" s="4" t="inlineStr"/>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr"/>
-      <c r="G78" s="4" t="inlineStr"/>
-    </row>
-    <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="n">
-        <v>75051</v>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 16000</t>
-        </is>
-      </c>
-      <c r="D79" s="4" t="inlineStr"/>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr"/>
-      <c r="G79" s="4" t="inlineStr"/>
-    </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="n">
-        <v>75052</v>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 32000</t>
-        </is>
-      </c>
-      <c r="D80" s="4" t="inlineStr"/>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F80" s="4" t="inlineStr"/>
-      <c r="G80" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G80"/>
+  <autoFilter ref="A1:G61"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -5124,25 +4357,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Show spell details in a right-hand panel and match the writeup files to the site.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -28,13 +28,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$G$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$G$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$G$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$G$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$G$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Xev Tests Fate'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Xev Tests Fate'!$A$1:$G$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Xev Tests Fate'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2222,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2549,72 +2549,103 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Arcing Slash</t>
+          <t>Tainted Affliction</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>75111</v>
+        <v>75110</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 700750 per Tick</t>
+          <t>Decrease Current Hit Points by 450000 per Tick</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Corrupting influence breaks your mind and body.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>The corrupting influence fades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Arcing Slash</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>75111</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 700750 per Tick</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>A quick slash causes you to bleed.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>The bleeding stops.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Wither</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="3" t="n">
         <v>75113</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000 per Tick
 Increase Corruption Counter by 30</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Corruption 30</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Corruption drains your life essence.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>The corruption dissipates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G12"/>
+  <autoFilter ref="A1:G13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2627,6 +2658,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -2647,7 +2679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3154,16 +3186,82 @@
       </c>
       <c r="G17" s="2" t="inlineStr"/>
     </row>
-    <row r="18" ht="96" customHeight="1">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>Stinking Miasma</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>12087</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 6000 per Tick
+Decrease Current Mana by 6000 per Tick
+Decrease Current Endurance by 1500 per Tick</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>You are engulfed in the miasma.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Your lungs clear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Stinking Miasma</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>75061</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 600000 per Tick
+Decrease Current Mana by 6000 per Tick
+Decrease Current Endurance by 1500 per Tick</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>You are engulfed in the miasma.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Your lungs clear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>Spirit Cleaver</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B20" s="3" t="n">
         <v>75024</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Decrease Attack by 500
 Decrease Current Hit Points by 122500 per Tick
@@ -3173,93 +3271,93 @@
 Increase Poison Counter by 297</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Poison 297</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>3m 36s</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>An invisible force of rage splits your soul in two.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>You feel whole again.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Soul Consumption</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B21" s="5" t="n">
         <v>75056</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 375000
 Decrease Current Mana by 2700</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Spear of Discord</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B22" s="3" t="n">
         <v>75057</v>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 425000
 Stun NPC for 10s (PC for 5.25s)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="96" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Wave of Rage</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B23" s="5" t="n">
         <v>75023</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Increase Spell Mana Cost by 1% to 50%
 Decrease Current Hit Points by 325000
@@ -3269,141 +3367,95 @@
 Increase Poison Counter by 396</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Poison 396</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Ikaav Venom</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
+      <c r="B24" s="3" t="n">
         <v>17057</v>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 7500
 Decrease Current Hit Points by 5000 per Tick
 Increase Poison Counter by 50</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Poison 50</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>10m</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Poison courses through your system after you were bitten.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>You sigh in relief as the poison fades away.</t>
         </is>
       </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Discord's Rebuke</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>75025</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 475000</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Chaos fills your mind and pains your soul.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Vis Percussio</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="n">
-        <v>48039</v>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use:</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Vis Percussio</t>
+          <t>Discord's Rebuke</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>75033</v>
+        <v>75025</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Decrease Current Hit Points by 475000</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr"/>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Chaos fills your mind and pains your soul.</t>
+        </is>
+      </c>
       <c r="G25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Vita Anuimis</t>
+          <t>Vis Percussio</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>48040</v>
+        <v>48039</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -3422,11 +3474,11 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Vita Anuimis</t>
+          <t>Vis Percussio</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>75034</v>
+        <v>75033</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -3442,268 +3494,314 @@
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28" ht="16" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>48040</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>75034</v>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use:</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
+      <c r="B30" s="3" t="n">
         <v>75031</v>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 222000 per Tick
 Decrease Melee Haste by 55%</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B31" s="3" t="n">
         <v>75039</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Decrease Melee Haste by 55% (v371, Incremental)
 Decrease Current Hit Points by 150000 per Tick</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B32" s="5" t="n">
         <v>75030</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 325000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="G32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B33" s="5" t="n">
         <v>75035</v>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Claustro Facultis</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n">
+      <c r="B34" s="3" t="n">
         <v>75036</v>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 275000
 Decrease Current Mana by 3510 (v417)</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Magic drains painfully from your body.</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Repenta Vitoris</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B35" s="5" t="n">
         <v>75032</v>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 456789 per Tick</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>A ball of electricity gathers around you.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Ignas Maxio</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B36" s="3" t="n">
         <v>75037</v>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 299000 per Tick
 Decrease Movement Speed by 65%</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Flames engulf you.</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="48" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Humas Maxio</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B37" s="5" t="n">
         <v>75038</v>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 444000
 Push Back 3 Units and Up 3 Units
 Stun for 2s</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>You are engulfed in grinding earth.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Gravitas Maxio</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B38" s="3" t="n">
         <v>75040</v>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
 Decrease Current Hit Points by 175000 per Tick</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>You feel the very earth pulling you apart.</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37" ht="64" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="64" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Resonating Beam</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B39" s="5" t="n">
         <v>75058</v>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Dispel Beneficial (100% Chance)
 Decrease Current Hit Points by 600000
@@ -3711,116 +3809,62 @@
 Decrease Current Endurance by 1850</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>You are hit by a powerful resonation.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="32" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Repulsion of the First Creation</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B40" s="3" t="n">
         <v>23056</v>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 10000
 Push Back 3 Units and Up 12 Units</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr"/>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>You are repulsed.</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr"/>
-    </row>
-    <row r="39" ht="32" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Repulsion of the First Creation</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B41" s="3" t="n">
         <v>75042</v>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 125000
 Push Back 3 Units and Up 12 Units</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40" ht="32" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>23077</v>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 12000</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="n">
-        <v>75053</v>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000</t>
-        </is>
-      </c>
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -3829,473 +3873,527 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>You are struck by the retribution of The First Creation.</t>
+          <t>You are repulsed.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
     </row>
-    <row r="42" ht="16" customHeight="1">
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Lava Elemental Protection</t>
+          <t>Retribution of the First Creation</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>23057</v>
+        <v>23077</v>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 100</t>
+          <t>Decrease Current Hit Points by 12000</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr"/>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
       <c r="G42" s="4" t="inlineStr"/>
     </row>
-    <row r="43" ht="16" customHeight="1">
+    <row r="43" ht="32" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Lava Elemental Protection</t>
+          <t>Retribution of the First Creation</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>23058</v>
+        <v>75053</v>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 200</t>
+          <t>Decrease Current Hit Points by 325000</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr"/>
       <c r="E43" s="4" t="inlineStr">
         <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>23057</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 100</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B44" s="5" t="n">
+      <c r="B45" s="3" t="n">
+        <v>23058</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 200</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
         <v>23059</v>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 300</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr"/>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr"/>
-      <c r="G44" s="4" t="inlineStr"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B45" s="5" t="n">
+      <c r="B47" s="3" t="n">
         <v>23060</v>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 400</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr"/>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
-      <c r="G45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n">
+      <c r="B48" s="3" t="n">
         <v>23061</v>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 500</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n">
+      <c r="B49" s="3" t="n">
         <v>23062</v>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 600</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="4" t="inlineStr"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B48" s="5" t="n">
+      <c r="B50" s="3" t="n">
         <v>23063</v>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 700</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr"/>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B49" s="5" t="n">
+      <c r="B51" s="3" t="n">
         <v>23064</v>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 800</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr"/>
-      <c r="G49" s="4" t="inlineStr"/>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B50" s="5" t="n">
+      <c r="B52" s="3" t="n">
         <v>23065</v>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 900</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr"/>
-      <c r="G50" s="4" t="inlineStr"/>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B51" s="5" t="n">
+      <c r="B53" s="3" t="n">
         <v>23066</v>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 1000</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F51" s="4" t="inlineStr"/>
-      <c r="G51" s="4" t="inlineStr"/>
-    </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B52" s="5" t="n">
+      <c r="B54" s="3" t="n">
         <v>75043</v>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 1000</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr"/>
-      <c r="E52" s="4" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr"/>
-      <c r="G52" s="4" t="inlineStr"/>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B53" s="5" t="n">
+      <c r="B55" s="3" t="n">
         <v>75044</v>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 2000</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr"/>
-      <c r="E53" s="4" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F53" s="4" t="inlineStr"/>
-      <c r="G53" s="4" t="inlineStr"/>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B54" s="5" t="n">
+      <c r="B56" s="3" t="n">
         <v>75045</v>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 3000</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr"/>
-      <c r="E54" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr"/>
-      <c r="G54" s="4" t="inlineStr"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B55" s="5" t="n">
+      <c r="B57" s="3" t="n">
         <v>75046</v>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 4000</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr"/>
-      <c r="E55" s="4" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F55" s="4" t="inlineStr"/>
-      <c r="G55" s="4" t="inlineStr"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n">
+      <c r="B58" s="3" t="n">
         <v>75047</v>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 5000</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr"/>
-      <c r="E56" s="4" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr"/>
-      <c r="G56" s="4" t="inlineStr"/>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B57" s="5" t="n">
+      <c r="B59" s="3" t="n">
         <v>75048</v>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 6000</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr"/>
-      <c r="E57" s="4" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B58" s="5" t="n">
+      <c r="B60" s="3" t="n">
         <v>75049</v>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 7000</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr"/>
-      <c r="E58" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr"/>
-      <c r="G58" s="4" t="inlineStr"/>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B59" s="5" t="n">
+      <c r="B61" s="3" t="n">
         <v>75050</v>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 8000</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr"/>
-      <c r="E59" s="4" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr"/>
-      <c r="G59" s="4" t="inlineStr"/>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B60" s="5" t="n">
+      <c r="B62" s="3" t="n">
         <v>75051</v>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 16000</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr"/>
-      <c r="G60" s="4" t="inlineStr"/>
-    </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B61" s="5" t="n">
+      <c r="B63" s="3" t="n">
         <v>75052</v>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 32000</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr"/>
-      <c r="E61" s="4" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr"/>
-      <c r="G61" s="4" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G61"/>
+  <autoFilter ref="A1:G63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -4357,6 +4455,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -4377,7 +4477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4429,38 +4529,761 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Barb of Tallon</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>68258</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 195000
+Decrease Melee Haste by 40%
+Decrease Movement Speed by 45%</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>3m 30s</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>The blood freezes in your veins.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Your blood thaws.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Barb of Tallon</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>68259</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 148908
+Stun for 1.5s up to Level 200</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Your veins incinerate.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Your blood cools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="64" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Barb of Tallon</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>68260</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 83672 per Tick
+Decrease Armor Class by 265 to 350, Based on Class
+Decrease Hate Generated by 200%
+Increase Disease Counter by 165</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Disease 165</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>60s</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Your stomach lurches and refuses to obey you.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>The plague leaves you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Barb of Tallon</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>68261</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Inhibit Spell Casting (Spell Silence)
+Melee and Skill Silence</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1 tick</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>The barb of Tallon sears your flesh.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>The poison leaves you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Barb of Tallon</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>68262</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Spell Haste by 30%
+Limit Type: Exclude Combat Skills
+Decrease Current Hit Points by 134727 per Tick</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Tallon's barbs tear through you.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>You break free of the barbs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Tallon's Power</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>68257</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Dispel (1000)
+Dispel (1000)
+Dispel (1000)
+Dispel (1000)
+Dispel (1000)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Your magic tears away as you're blasted upward and flung back.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sword Storm</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>68263</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1072500</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Whirling blades rip into you as the storm engulfs you.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
           <t>Protection of Zek</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>68235</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Decrease Spell Damage Taken by 1% to 20% (v296, Before Crit)
 Decrease Damage Shield Taken by 20%
 Decrease Hit Damage Taken by 20%</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>5m</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3" ht="64" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Axe Sweep</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>49945</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Melee Attack for 79100 with 10000% Accuracy Mod</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>You are struck by an axe.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Axe Sweep</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>68236</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1300000</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>You are nearly bisected by Eriak Zek's axe.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Axe Sweep</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>74954</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 682500</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>You are nearly bisected by Eriak Zek's axe.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Blacksmith's Corrosion</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>68237</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Armor Class by 331 to 438, Based on Class</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Corrosive energy melts through your protection.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>The corrosion ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Blacksmith's Corrosion</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>74955</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Armor Class by 166 to 219, Based on Class</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Corrosive energy melts through your protection.</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>The corrosion ends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Aggressive Punch</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>68238</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 650000
+Stun for 1.5s</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>A katar?backed punch rips through your guard.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Aggressive Punch</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>74956</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 341250
+Stun for 1.5s</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>A katar-backed punch rips through your guard.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Eriak's Fortification</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>68239</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Absorb Spell Damage: 50%
+Absorb Melee Damage: 50%
+Absorb DoT Damage: 50%</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Confining Bonds</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>68240</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Root
+Decrease Current Hit Points by 195000 per Tick</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Eriak Zek's bonds lock your feet to the ground.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Eriak Zek's bindings loosen their grip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Confining Bonds</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>74957</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Root
+Decrease Current Hit Points by 85313 per Tick</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Eriak Zek's bonds lock your feet to the ground.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Eriak Zek's bindings loosen their grip.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Spear of Zek</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>68241</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1755000</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>The Spear of Zek drives straight through you.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Spear of Zek</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>74958</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 341250</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>The Spear of Zek drives straight through you.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Rapid Shanks</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>68243</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 195000 per Tick</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>A blur of flashing blades whirls past--one cuts into you.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Rapid Shanks</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>74960</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Summon Pet:
+Decrease Current Hit Points by 85313</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>A blur of flashing blades whirls past--one cuts into you.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Assassination of Zek</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>68242</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 9000000000</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>A perfect backstab ends you instantly.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Assassination of Zek</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>74959</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 9000000000</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>A perfect backstab ends you instantly.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Razor Armor</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>68251</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Add Defensive Proc:</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Razor Armor</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>74965</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Add Defensive Proc:</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="64" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>Eriak's Doom</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B28" s="5" t="n">
         <v>68247</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Cast on Duration Fade:
 Increase Curse Counter by 99
@@ -4468,32 +5291,116 @@
 Limit Spells:</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Curse 99</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>Eriak's Doom binds you, ruin coming when its time ends.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>Eriak's Doom fades.</t>
         </is>
       </c>
     </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Doom of the Blacksmith</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>68265</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 9000000000</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>You have been struck down by the Doom of Eriak.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="64" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Greedy Repercussions</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>68248</v>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Increase Spell Mana Cost by 1% to 30%
+Decrease Melee Haste by 30% (v371, Incremental)
+Decrease Current Hit Points by 1 per Tick
+Decrease Current Hit Points by 1</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>8 ticks</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>A greedy force wraps around you, taxing your every action.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G30"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -4514,7 +5421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4742,62 +5649,133 @@
       </c>
       <c r="G7" s="4" t="inlineStr"/>
     </row>
-    <row r="8" ht="16" customHeight="1">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lucky Boon</t>
+          <t>Forced Transfer</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>75083</v>
+        <v>75077</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Increase Max Hit Points by 45%</t>
+          <t>Decrease Healing Taken by 1% to 75% (v393)
+Cast on Limit Match:</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1m 12s</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>You feel the boon of luck.</t>
-        </is>
-      </c>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Unlucky Hindrance</t>
+          <t>Lucksworn Empower</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>75084</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 200000</t>
-        </is>
-      </c>
+        <v>75080</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Crushing Laxity</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>75082</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 750000 per Tick
+Decrease Movement Speed by 40%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>The weight of your misstep crushes you.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Lucky Boon</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>75083</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Increase Max Hit Points by 45%</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>1m 12s</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>You feel the boon of luck.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Unlucky Hindrance</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>75084</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 200000</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>You feel the ire of luck.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -4807,6 +5785,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Fill in the spells Maddening Influence casts when cured or when it fades.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -2285,8 +2285,8 @@
           <t>Decrease Current Hit Points by 600600 per Tick
 Increase Corruption Counter by 24
 Increase Attack by 25
-Cast if Cured:
-Cast on Duration Fade:</t>
+Cast if Cured: Corrupting Pulse
+Cast on Duration Fade: Ensorcel Psyche</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Update Stronger Together's Land on Other text and show that line in the spreadsheet.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -18,23 +18,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xev Tests Fate" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Siren Sisters'!$A$1:$G$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Siren Sisters'!$A$1:$H$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Siren Sisters'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dipuc'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dipuc'!$A$1:$H$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$G$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$63</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$G$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$H$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Xev Tests Fate'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Xev Tests Fate'!$A$1:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Xev Tests Fate'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -487,7 +487,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,6 +524,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -554,7 +560,8 @@
           <t>A soothing song envelops you.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>You no longer feel the soothing song.</t>
         </is>
@@ -587,7 +594,8 @@
           <t>Your throat tightens, making it impossible to speak.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Your throat loosens.</t>
         </is>
@@ -620,7 +628,8 @@
           <t>Words of power course through you.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>You no longer feel empowered.</t>
         </is>
@@ -652,7 +661,8 @@
           <t>Your body tightens and freezes in place.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Your muscles loosen and respond.</t>
         </is>
@@ -685,7 +695,8 @@
           <t>A gentle melody uplifts you.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>You no longer feel uplifted.</t>
         </is>
@@ -717,14 +728,15 @@
           <t>An immense weight slows your movement</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>The weight lifts.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:H7"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -752,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -761,7 +773,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -797,6 +810,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -827,6 +845,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -854,6 +873,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -877,7 +897,12 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Target is filled with scorn.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -905,7 +930,8 @@
           <t>A painful weight settles in on your chest.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>The weight lifts.</t>
         </is>
@@ -940,9 +966,10 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:H6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -969,7 +996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -978,7 +1005,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1014,6 +1042,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -1044,6 +1077,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -1071,7 +1105,8 @@
           <t>You draw energy from the surrounding area.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>You no longer feel empowered.</t>
         </is>
@@ -1103,7 +1138,8 @@
           <t>Your attacks seem faster.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Your attacks return to normal.</t>
         </is>
@@ -1136,7 +1172,8 @@
           <t>A protective barrier covers you.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>The protective barrier fades.</t>
         </is>
@@ -1167,7 +1204,8 @@
           <t>A soothing energy fills you.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>The soothing energy fades.</t>
         </is>
@@ -1198,7 +1236,8 @@
           <t>Thorned shackles wrap around your legs.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>The shackles shrivel and break.</t>
         </is>
@@ -1230,7 +1269,8 @@
           <t>Your attacks and spells feel weaker.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>You feel invigorated again.</t>
         </is>
@@ -1261,7 +1301,8 @@
           <t>Flowering buds spring from your skin.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>The flowers bloom and fall away.</t>
         </is>
@@ -1292,7 +1333,8 @@
           <t>Sapping runes cover your body.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>The runes disappear.</t>
         </is>
@@ -1322,6 +1364,11 @@
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr">
         <is>
+          <t>Targetwraps herself in sharp barbs.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
           <t>The barbs fall away.</t>
         </is>
       </c>
@@ -1352,7 +1399,8 @@
           <t>Your body moves on its own.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>You regain control of your body.</t>
         </is>
@@ -1384,6 +1432,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1406,7 +1455,12 @@
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>Targetis unable to form words of encouragement.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
     </row>
     <row r="15" ht="96" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -1436,7 +1490,8 @@
           <t>Your inner fire grows to an inferno.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Your inner fire dims.</t>
         </is>
@@ -1469,14 +1524,15 @@
           <t>Your spirit is crushed.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>You refocus on the fight.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:H16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1513,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1522,7 +1578,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1558,6 +1615,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -1592,7 +1654,8 @@
           <t>You inhale a potent toxin that burns your lungs.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>The poison runs its course.</t>
         </is>
@@ -1625,6 +1688,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1653,6 +1717,7 @@
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1681,6 +1746,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -1708,6 +1774,7 @@
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -1735,6 +1802,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1762,7 +1830,8 @@
           <t>The razor sharp jaws of the trap cut into your leg.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Your wounds close.</t>
         </is>
@@ -1795,7 +1864,8 @@
           <t>Moruuk's blow rattles you, slowing your reactions.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>You shake off the attack.</t>
         </is>
@@ -1822,7 +1892,12 @@
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Target's attacks become faster and more aggressive.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1851,6 +1926,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="80" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1881,6 +1957,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -1911,9 +1988,10 @@
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:H13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -1947,7 +2025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1956,7 +2034,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1992,6 +2071,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -2022,6 +2106,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -2049,6 +2134,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -2076,7 +2162,8 @@
           <t>Taurlton's gaze rests uneasily on you.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Taurlton's gaze is broken by the falling debris.</t>
         </is>
@@ -2109,6 +2196,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -2136,6 +2224,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -2163,6 +2252,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -2191,9 +2281,10 @@
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:H8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2222,7 +2313,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2231,7 +2322,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2266,6 +2358,11 @@
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Wear off</t>
         </is>
@@ -2304,7 +2401,8 @@
           <t>Whispers of dark thoughts intrude your mind.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>The whispers dissipate.</t>
         </is>
@@ -2336,6 +2434,7 @@
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -2362,7 +2461,8 @@
           <t>The mist clings to your throat, preventing you from speaking.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>The mist clears, you can speak again.</t>
         </is>
@@ -2394,7 +2494,8 @@
           <t>A piercing shriek rattles your mind.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Your mind clears</t>
         </is>
@@ -2426,6 +2527,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -2452,7 +2554,8 @@
           <t>Psychic energy shatters your spirit.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>You pull yourself together.</t>
         </is>
@@ -2485,6 +2588,7 @@
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -2511,7 +2615,8 @@
           <t>Vazaelle's judgement makes it difficult to defend yourself.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>You can defend yourself again.</t>
         </is>
@@ -2545,6 +2650,7 @@
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -2571,7 +2677,8 @@
           <t>Corrupting influence breaks your mind and body.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>The corrupting influence fades.</t>
         </is>
@@ -2602,7 +2709,8 @@
           <t>A quick slash causes you to bleed.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>The bleeding stops.</t>
         </is>
@@ -2638,14 +2746,15 @@
           <t>Corruption drains your life essence.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>The corruption dissipates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:H13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2679,7 +2788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2688,7 +2797,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2724,6 +2834,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -2750,6 +2865,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -2773,6 +2889,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -2799,7 +2916,12 @@
           <t>You feel a tugging at your soul.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Target staggers.</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2826,7 +2948,12 @@
           <t>You feel a tugging at your soul.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Target staggers.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -2861,6 +2988,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -2895,6 +3023,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -2923,6 +3052,11 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
+          <t>Target's body begins to splurt.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
           <t>Your body stops splurting.</t>
         </is>
       </c>
@@ -2954,6 +3088,11 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
+          <t>Target's body begins to splurt.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
           <t>Your body stops splurting.</t>
         </is>
       </c>
@@ -2983,7 +3122,12 @@
           <t>You have been burnt by a wizard's blast of self-immolation.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Target has been burnt by a wizard's blast of self-immolation.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -3010,7 +3154,12 @@
           <t>You have been burnt by a wizard's blast of self-immolation.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Target has been burnt by a wizard's blast of self-immolation.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -3038,7 +3187,12 @@
           <t>Sharpened horns gore your flesh.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Target is gored by sharpened horns.</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -3066,7 +3220,12 @@
           <t>Sharpened horns gore your flesh.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Target is gored by sharpened horns.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -3094,7 +3253,12 @@
           <t>You are slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Target is slain by a mighty cleave.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -3122,7 +3286,12 @@
           <t>You are slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Target is slain by a mighty cleave.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="64" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -3154,6 +3323,11 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
+          <t>Target looks somewhat uncomfortable.</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
           <t>Your vulnerability fades.</t>
         </is>
       </c>
@@ -3184,7 +3358,12 @@
           <t>You are filled with a sense of bitter spite.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Target is knocked back.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
@@ -3215,6 +3394,11 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
+          <t>Target is caught in the miasma.</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
           <t>Your lungs clear.</t>
         </is>
       </c>
@@ -3247,6 +3431,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Target is caught in the miasma.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Your lungs clear.</t>
         </is>
@@ -3288,6 +3477,11 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
+          <t>Target's soul splits in two.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
           <t>You feel whole again.</t>
         </is>
       </c>
@@ -3318,7 +3512,12 @@
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Target staggers for a moment.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -3346,7 +3545,12 @@
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Target is pierced by the spear of discord.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="96" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -3382,7 +3586,12 @@
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Target succumbs to the temptation of rage.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -3417,6 +3626,11 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
+          <t>Target Poison courses through their system after they were bitten.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
           <t>You sigh in relief as the poison fades away.</t>
         </is>
       </c>
@@ -3446,7 +3660,12 @@
           <t>Chaos fills your mind and pains your soul.</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Target jerks and spasms in pain.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -3470,6 +3689,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -3493,6 +3713,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr"/>
       <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -3516,6 +3737,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="4" t="inlineStr"/>
+      <c r="H28" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -3539,6 +3761,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -3567,6 +3790,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
     </row>
     <row r="31" ht="32" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
@@ -3595,6 +3819,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -3623,6 +3848,7 @@
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
+      <c r="H32" s="4" t="inlineStr"/>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -3651,6 +3877,7 @@
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
     </row>
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
@@ -3679,6 +3906,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -3706,6 +3934,7 @@
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr"/>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
@@ -3734,6 +3963,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -3763,6 +3993,7 @@
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
     </row>
     <row r="38" ht="32" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
@@ -3791,6 +4022,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
     </row>
     <row r="39" ht="64" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
@@ -3821,6 +4053,7 @@
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
     </row>
     <row r="40" ht="32" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
@@ -3848,7 +4081,12 @@
           <t>You are repulsed.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Target is repulsed.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
     </row>
     <row r="41" ht="32" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -3876,7 +4114,12 @@
           <t>You are repulsed.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Target is repulsed.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
     </row>
     <row r="42" ht="32" customHeight="1">
       <c r="A42" s="4" t="inlineStr">
@@ -3903,7 +4146,12 @@
           <t>You are struck by the retribution of The First Creation.</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Target is struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="32" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
@@ -3930,7 +4178,12 @@
           <t>You are struck by the retribution of The First Creation.</t>
         </is>
       </c>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Target is struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -3954,6 +4207,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
@@ -3977,6 +4231,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -4000,6 +4255,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
@@ -4023,6 +4279,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
@@ -4046,6 +4303,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
@@ -4069,6 +4327,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr"/>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -4092,6 +4351,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
@@ -4115,6 +4375,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -4138,6 +4399,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr"/>
       <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
@@ -4161,6 +4423,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr"/>
       <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
     </row>
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -4184,6 +4447,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr"/>
       <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
     </row>
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
@@ -4207,6 +4471,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr"/>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -4230,6 +4495,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
@@ -4253,6 +4519,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr"/>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
@@ -4276,6 +4543,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
@@ -4299,6 +4567,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr"/>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -4322,6 +4591,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -4345,6 +4615,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr"/>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
@@ -4368,6 +4639,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
@@ -4391,9 +4663,10 @@
       </c>
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G63"/>
+  <autoFilter ref="A1:H63"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -4477,7 +4750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4486,7 +4759,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4522,6 +4796,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -4555,6 +4834,11 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Target has been struck by a huge frozen arrow.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Your blood thaws.</t>
         </is>
       </c>
@@ -4586,6 +4870,11 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Target screams as the arrow ignites their blood.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Your blood cools.</t>
         </is>
@@ -4625,6 +4914,11 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>Target struggles to stay on their feet as the disease infests them.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>The plague leaves you.</t>
         </is>
       </c>
@@ -4656,6 +4950,11 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Target has been poisoned by Tallon's barb.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>The poison leaves you.</t>
         </is>
@@ -4689,6 +4988,11 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Target is struck by a hail of barbs.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>You break free of the barbs.</t>
         </is>
@@ -4723,7 +5027,12 @@
           <t>Your magic tears away as you're blasted upward and flung back.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Target is thrown back and stripped of buffs.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -4750,7 +5059,12 @@
           <t>Whirling blades rip into you as the storm engulfs you.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Target is slashed by blades</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -4775,7 +5089,12 @@
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Target is protected by the power of the Zek family.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -4802,7 +5121,12 @@
           <t>You are struck by an axe.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Target is struck by an axe.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -4829,7 +5153,12 @@
           <t>You are nearly bisected by Eriak Zek's axe.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Target is nearly bisected by Eriak Zek's axe.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -4856,7 +5185,12 @@
           <t>You are nearly bisected by Eriak Zek's axe.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Target is nearly bisected by Eriak Zek's axe.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -4885,6 +5219,11 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
+          <t>Target's protection melts.</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
           <t>The corrosion ends.</t>
         </is>
       </c>
@@ -4916,6 +5255,11 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
+          <t>Target's protection melts.</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
           <t>The corrosion ends.</t>
         </is>
       </c>
@@ -4946,7 +5290,12 @@
           <t>A katar?backed punch rips through your guard.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Target is punched with a Katar.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -4974,7 +5323,12 @@
           <t>A katar-backed punch rips through your guard.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Target is punched with a Katar.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -4999,7 +5353,12 @@
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Target is Fortified.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -5029,6 +5388,11 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
+          <t>Target's feet are bound to the ground.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
           <t>Eriak Zek's bindings loosen their grip.</t>
         </is>
       </c>
@@ -5061,6 +5425,11 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
+          <t>Target's feet are bound to the ground.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
           <t>Eriak Zek's bindings loosen their grip.</t>
         </is>
       </c>
@@ -5090,7 +5459,12 @@
           <t>The Spear of Zek drives straight through you.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Target is skewered by the Spear of Zek.</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
@@ -5117,7 +5491,12 @@
           <t>The Spear of Zek drives straight through you.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Target is skewered by the Spear of Zek.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -5144,7 +5523,12 @@
           <t>A blur of flashing blades whirls past--one cuts into you.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Target is stabbed.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -5172,7 +5556,12 @@
           <t>A blur of flashing blades whirls past--one cuts into you.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Target is stabbed.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -5199,7 +5588,12 @@
           <t>A perfect backstab ends you instantly.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Target is killed by a backstab.</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -5226,7 +5620,12 @@
           <t>A perfect backstab ends you instantly.</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Target is killed by a backstab.</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -5249,7 +5648,12 @@
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Target is protected by sharply reactive armor.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
@@ -5272,7 +5676,12 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Target is protected by sharply reactive armor.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
     </row>
     <row r="28" ht="64" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
@@ -5308,6 +5717,11 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
+          <t>Target is promised ruin and doom.</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
           <t>Eriak's Doom fades.</t>
         </is>
       </c>
@@ -5337,7 +5751,12 @@
           <t>You have been struck down by the Doom of Eriak.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Target is struck by the Doom of Eriak</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
     </row>
     <row r="30" ht="64" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
@@ -5367,10 +5786,15 @@
           <t>A greedy force wraps around you, taxing your every action.</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Target is wrapped by greed.</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G30"/>
+  <autoFilter ref="A1:H30"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -5421,7 +5845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -5430,7 +5854,8 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5466,6 +5891,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Land on Other</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Wear off</t>
         </is>
       </c>
@@ -5496,7 +5926,8 @@
           <t>Your mind and muscles feel sluggish and are slow to respond.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Your body and mind start responding again.</t>
         </is>
@@ -5529,7 +5960,8 @@
           <t>You are overwhelmed with fear.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>You regain control of your senses.</t>
         </is>
@@ -5561,6 +5993,7 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -5588,6 +6021,7 @@
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -5615,7 +6049,8 @@
           <t>Fate can give and take; this time it gave.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Fate's gift fades.</t>
         </is>
@@ -5648,6 +6083,7 @@
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -5672,6 +6108,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -5691,6 +6128,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -5719,6 +6157,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -5746,6 +6185,7 @@
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -5773,9 +6213,10 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G12"/>
+  <autoFilter ref="A1:H12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>

</xml_diff>

<commit_message>
Add the Siren Sisters anger pulses the writeup already named.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -18,7 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xev Tests Fate" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Siren Sisters'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Siren Sisters'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Siren Sisters'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Dipuc'!$A$1:$H$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -567,176 +567,530 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>Shrill Chorus</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>75161</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 110000</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>A shrill song rattles you to the core.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Shrill Chorus</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>75162</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 275000</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>A shrill song rattles you to the core.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Shrill Chorus</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>75163</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 425000</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>A shrill song rattles you to the core.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="64" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Shrill Chorus</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>75164</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 550000
+Decrease Current Hit Points by 225000 per Tick
+Inhibit Spell Casting (Spell Silence)
+Melee and Skill Silence</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>A shrill song rattles you to the core and takes your voice.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Your voice returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Lingering Hymn</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B7" s="3" t="n">
         <v>75165</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000 per Tick
 Inhibit Spell Casting (Spell Silence)
 Melee and Skill Silence</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Your throat tightens, making it impossible to speak.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Your throat loosens.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="64" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Empowering Rhetoric</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>75166</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Decrease Spell and DoT Damage Taken by 1% to 50% (v483, After Crit)
 Limit Spells:
 Limit Type: Include Non-Focusable</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>1 tick</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Words of power course through you.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>You no longer feel empowered.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cutting Verse</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>75167</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 110000</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>The words cut deep.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Cutting Verse</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>75168</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 275000</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>The words cut deep.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Cutting Verse</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>75169</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 425000</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>The words cut deep.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cutting Verse</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>75170</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 750000
+Stun for 12s</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>The words cut deep and your body stops responding.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Your body begins to respond.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Biting Sonnet</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>75171</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000
 Stun for 6s</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Your body tightens and freezes in place.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Your muscles loosen and respond.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="64" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Tranquil Rhythm</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B14" s="3" t="n">
         <v>75172</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Decrease Spell and DoT Damage Taken by 1% to 50% (v483, After Crit)
 Limit Spells:
 Limit Type: Include Non-Focusable</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1 tick</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>A gentle melody uplifts you.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>You no longer feel uplifted.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Discordant Melody</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>75173</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 110000</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>A cacophonous burst crushes you.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Discordant Melody</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>75174</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 275000</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>A cacophonous burst crushes you.</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Discordant Melody</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>75175</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 425000</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>A cacophonous burst crushes you.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Discordant Melody</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>75176</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 550000
+Decrease Current Hit Points by 225000 per Tick
+Decrease Movement Speed by 350%</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>A cacophonous burst crushes you, slowing your movement.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Your movement is no longer slowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Cacophonous Note</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B19" s="3" t="n">
         <v>75177</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 440000 per Tick
 Decrease Movement Speed by 180%</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>An immense weight slows your movement</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>The weight lifts.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -744,6 +1098,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Update the site from the latest beta forum posts and spell pages.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -545,7 +545,7 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Decrease Spell and DoT Damage Taken by 1% to 50% (v483, After Crit)
-Limit Spells:
+Limit Spells: Discordant Melody I
 Limit Type: Include Non-Focusable</t>
         </is>
       </c>
@@ -732,7 +732,7 @@
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Decrease Spell and DoT Damage Taken by 1% to 50% (v483, After Crit)
-Limit Spells:
+Limit Spells: Shrill Chorus I
 Limit Type: Include Non-Focusable</t>
         </is>
       </c>
@@ -916,7 +916,7 @@
       <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Decrease Spell and DoT Damage Taken by 1% to 50% (v483, After Crit)
-Limit Spells:
+Limit Spells: Cutting Verse I
 Limit Type: Include Non-Focusable</t>
         </is>
       </c>
@@ -2514,7 +2514,7 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 500500 per Tick
-Cast on Duration Fade:</t>
+Cast on Duration Fade: Black Listed</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
@@ -2547,7 +2547,7 @@
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600500
-Cast on Fade:</t>
+Cast on Fade: Black Listed</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
@@ -4044,7 +4044,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr"/>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Cast on Skill Use:</t>
+          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr"/>
@@ -6004,7 +6004,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Add Defensive Proc:</t>
+          <t>Add Defensive Proc: Razor Slash with 1000% Rate Mod</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
@@ -6032,7 +6032,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Add Defensive Proc:</t>
+          <t>Add Defensive Proc: Razor Slash with 1000% Rate Mod</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
@@ -6060,10 +6060,10 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Cast on Duration Fade:
+          <t>Cast on Duration Fade: Doom of the Blacksmith
 Increase Curse Counter by 99
 Increase Spell Damage Taken by 1 (v297, Before Crit)
-Limit Spells:</t>
+Limit Spells: Greedy Repercussions</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -6463,7 +6463,7 @@
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Decrease Healing Taken by 1% to 75% (v393)
-Cast on Limit Match:</t>
+Cast on Limit Match: Transfer In Progress</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Remove older spell copies that are not used on these raids.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -24,13 +24,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$H$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$43</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$H$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
@@ -1935,7 +1935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2034,23 +2034,23 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>52393</v>
+        <v>75134</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 135165 per Tick
-Decrease Current Hit Points by 111111</t>
+          <t>Decrease Current Hit Points by 600600
+Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>3 ticks</t>
+          <t>2 ticks</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>The griffin rakes with its back claws.</t>
+          <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>75134</v>
+        <v>75135</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -2085,30 +2085,29 @@
       <c r="G4" s="4" t="inlineStr"/>
       <c r="H4" s="4" t="inlineStr"/>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>75135</v>
+        <v>75151</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 600600
-Inhibit Spell Casting (Spell Silence)</t>
+          <t>Fling</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>2 ticks</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>The manticore's claws rake across your flesh.</t>
+          <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
@@ -2121,7 +2120,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>75151</v>
+        <v>75152</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -2142,168 +2141,140 @@
       <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Rake</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>75152</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Fling</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>The manticore's claws strike throws you back.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Lockjaw Trap</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B7" s="3" t="n">
         <v>75137</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Root</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>The razor sharp jaws of the trap cut into your leg.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Your wounds close.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Slow Your Roll</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B8" s="5" t="n">
         <v>75138</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 750000
 Decrease Melee Haste by 10% (v371, Incremental)
 Increase Cast Time by 1s</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Moruuk's blow rattles you, slowing your reactions.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>You shake off the attack.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Stronger Together</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B9" s="3" t="n">
         <v>75141</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Increase Melee Haste by 25%</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Target's attacks become faster and more aggressive.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Taking Your Stuff</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B10" s="5" t="n">
         <v>75140</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Mana by 0.1% of Total Mana, Max: 0
 Decrease Current Endurance by 0.1% of Total Endurance, Max: 0</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>You feel drained.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Aura of Greed</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B11" s="3" t="n">
         <v>75147</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2311,30 +2282,30 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>The weight of your poverty takes its toll.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Aura of Poverty</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B12" s="5" t="n">
         <v>75148</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2342,22 +2313,22 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>The weight of your greed takes its toll.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H12"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2370,7 +2341,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -3154,7 +3124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3216,11 +3186,11 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>12196</v>
+        <v>75003</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 20000</t>
+          <t>Decrease Current Hit Points by 200000</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
@@ -3234,138 +3204,47 @@
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Power of the Synarcana</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>75003</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 200000</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Lethal Lifetap</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>75004</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 450000</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Lethal Lifetap</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>12204</v>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 45000</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>You feel a tugging at your soul.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Target staggers.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Lethal Lifetap</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>75004</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 450000</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>You feel a tugging at your soul.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Target staggers.</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="64" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="64" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Spreading Evil</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
-        <v>12209</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 35000
-Decrease Current Hit Points by 10000 per Tick
-Decrease Melee Haste by 70% (v371, Incremental)
-Increase Corruption Counter by 20</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Corruption 20</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Evil swarms over you and seethes in the air around you</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="64" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Spreading Evil</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
+      <c r="B4" s="3" t="n">
         <v>75005</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000
 Decrease Current Hit Points by 100000 per Tick
@@ -3373,302 +3252,168 @@
 Increase Corruption Counter by 20</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Corruption 20</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Evil swarms over you and seethes in the air around you</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Splart</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>19035</v>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="B5" s="5" t="n">
+        <v>75007</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 63 per Tick (Growing @ 64/Tick)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>2m</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Your body begins to splurt.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Target's body begins to splurt.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Your body stops splurting.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Splart</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>75007</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 63 per Tick (Growing @ 64/Tick)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>2m</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Your body begins to splurt.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Target's body begins to splurt.</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Your body stops splurting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Self-Immolation</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
-        <v>19920</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 8915</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="B6" s="3" t="n">
+        <v>75009</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 82994</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>You have been burnt by a wizard's blast of self-immolation.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Target has been burnt by a wizard's blast of self-immolation.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Self-Immolation</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>75009</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 82994</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>You have been burnt by a wizard's blast of self-immolation.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Target has been burnt by a wizard's blast of self-immolation.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Minotaur Gore</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>13023</v>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 50000</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Sharpened horns gore your flesh.</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Target is gored by sharpened horns.</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Minotaur Gore</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
+      <c r="B7" s="5" t="n">
         <v>75013</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 650000</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Sharpened horns gore your flesh.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Target is gored by sharpened horns.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Decapitating Chop</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
-        <v>7234</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Feign Death (1% Chance)
-Decrease Current Hit Points by 100000</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>You are slain by a mighty cleave.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Target is slain by a mighty cleave.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Decapitating Chop</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
+      <c r="B8" s="3" t="n">
         <v>75014</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 4000000000</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>You are slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Target is slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="64" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Malaise</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B9" s="5" t="n">
         <v>110</v>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Decrease Cold Resist by 20
 Decrease Magic Resist by 20
@@ -3676,147 +3421,109 @@
 Decrease Fire Resist by 20</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>14m</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>You feel somewhat vulnerable.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Target looks somewhat uncomfortable.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Your vulnerability fades.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="10" ht="64" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Spite</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B10" s="3" t="n">
         <v>40778</v>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 25000 per Tick (Scales, Base Level: 105)
 Decrease Current Mana by 10000 per Tick (Scales, Base Level: 105) (v417)</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>You are filled with a sense of bitter spite.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Target is knocked back.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Stinking Miasma</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>12087</v>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 6000 per Tick
-Decrease Current Mana by 6000 per Tick
-Decrease Current Endurance by 1500 per Tick</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>3 ticks</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>You are engulfed in the miasma.</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Target is caught in the miasma.</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Your lungs clear.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Stinking Miasma</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
+      <c r="B11" s="5" t="n">
         <v>75061</v>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600000 per Tick
 Decrease Current Mana by 6000 per Tick
 Decrease Current Endurance by 1500 per Tick</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>You are engulfed in the miasma.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>Target is caught in the miasma.</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Your lungs clear.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="96" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="12" ht="96" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Spirit Cleaver</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B12" s="3" t="n">
         <v>75024</v>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Decrease Attack by 500
 Decrease Current Hit Points by 122500 per Tick
@@ -3826,108 +3533,108 @@
 Increase Poison Counter by 297</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Poison 297</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>3m 36s</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>An invisible force of rage splits your soul in two.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Target's soul splits in two.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>You feel whole again.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Soul Consumption</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>75056</v>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 375000
 Decrease Current Mana by 2700</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Target staggers for a moment.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Spear of Discord</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B14" s="3" t="n">
         <v>75057</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 425000
 Stun NPC for 10s (PC for 5.25s)</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Target is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="96" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Wave of Rage</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B15" s="5" t="n">
         <v>75023</v>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Increase Spell Mana Cost by 1% to 50%
 Decrease Current Hit Points by 325000
@@ -3937,82 +3644,298 @@
 Increase Poison Counter by 396</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Poison 396</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Target succumbs to the temptation of rage.</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Ikaav Venom</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B16" s="3" t="n">
         <v>17057</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 7500
 Decrease Current Hit Points by 5000 per Tick
 Increase Poison Counter by 50</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Poison 50</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>10m</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Poison courses through your system after you were bitten.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Target Poison courses through their system after they were bitten.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>You sigh in relief as the poison fades away.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Discord's Rebuke</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>75025</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 475000</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Chaos fills your mind and pains your soul.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Target jerks and spasms in pain.</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Vis Percussio</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>48039</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Vis Percussio</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>75033</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>48040</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>75034</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Vita Tardius</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>75031</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 222000 per Tick
+Decrease Melee Haste by 55%</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Your body convulses as electricity runs through you.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Vita Tardius</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>75039</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Melee Haste by 55% (v371, Incremental)
+Decrease Current Hit Points by 150000 per Tick</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Your body convulses as electricity runs through you.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Claustro Vitoris</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>75030</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 325000
+Stun for 1s</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>You are shocked!</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Discord's Rebuke</t>
+          <t>Claustro Vitoris</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>75025</v>
+        <v>75035</v>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 475000</t>
+          <t>Decrease Current Hit Points by 350000
+Stun for 1s</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr"/>
@@ -4023,383 +3946,167 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Chaos fills your mind and pains your soul.</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Target jerks and spasms in pain.</t>
-        </is>
-      </c>
+          <t>You are shocked!</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr"/>
       <c r="H25" s="4" t="inlineStr"/>
     </row>
-    <row r="26" ht="16" customHeight="1">
+    <row r="26" ht="32" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Vis Percussio</t>
+          <t>Claustro Facultis</t>
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>48039</v>
+        <v>75036</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
+          <t>Decrease Current Hit Points by 275000
+Decrease Current Mana by 3510 (v417)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Magic drains painfully from your body.</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr"/>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Vis Percussio</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="n">
-        <v>75033</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>48040</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr"/>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>75034</v>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>75031</v>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 222000 per Tick
-Decrease Melee Haste by 55%</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Vita Tardius</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="n">
-        <v>75039</v>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Melee Haste by 55% (v371, Incremental)
-Decrease Current Hit Points by 150000 per Tick</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>5 ticks</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Your body convulses as electricity runs through you.</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>75030</v>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Claustro Vitoris</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>75035</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 350000
-Stun for 1s</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>You are shocked!</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Claustro Facultis</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>75036</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 275000
-Decrease Current Mana by 3510 (v417)</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Magic drains painfully from your body.</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Repenta Vitoris</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
+      <c r="B27" s="5" t="n">
         <v>75032</v>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 456789 per Tick</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>A ball of electricity gathers around you.</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-    </row>
-    <row r="36" ht="32" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Ignas Maxio</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B28" s="3" t="n">
         <v>75037</v>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 299000 per Tick
 Decrease Movement Speed by 65%</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Flames engulf you.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="48" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Humas Maxio</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B29" s="5" t="n">
         <v>75038</v>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 444000
 Push Back 3 Units and Up 3 Units
 Stun for 2s</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr"/>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>You are engulfed in grinding earth.</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr"/>
-      <c r="H37" s="4" t="inlineStr"/>
-    </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Gravitas Maxio</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B30" s="3" t="n">
         <v>75040</v>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
 Decrease Current Hit Points by 175000 per Tick</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>You feel the very earth pulling you apart.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="64" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="64" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Resonating Beam</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B31" s="5" t="n">
         <v>75058</v>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Dispel Beneficial (100% Chance)
 Decrease Current Hit Points by 600000
@@ -4407,632 +4114,327 @@
 Decrease Current Endurance by 1850</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr"/>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>You are hit by a powerful resonation.</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr"/>
-      <c r="H39" s="4" t="inlineStr"/>
-    </row>
-    <row r="40" ht="32" customHeight="1">
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Repulsion of the First Creation</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>75042</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 125000
+Push Back 3 Units and Up 12 Units</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>You are repulsed.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Target is repulsed.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Retribution of the First Creation</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>75053</v>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 325000</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Target is struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>75043</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 1000</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>75044</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 2000</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>75045</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 3000</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>75046</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 4000</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>75047</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 5000</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>75048</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 6000</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Repulsion of the First Creation</t>
+          <t>Lava Elemental Protection</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>23056</v>
+        <v>75049</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 10000
-Push Back 3 Units and Up 12 Units</t>
+          <t>Increase Damage Shield by 7000</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Target is repulsed.</t>
-        </is>
-      </c>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="16" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Repulsion of the First Creation</t>
+          <t>Lava Elemental Protection</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>75042</v>
+        <v>75050</v>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 125000
-Push Back 3 Units and Up 12 Units</t>
+          <t>Increase Damage Shield by 8000</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Target is repulsed.</t>
-        </is>
-      </c>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
     </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="n">
-        <v>23077</v>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 12000</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr"/>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>Target is struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-    </row>
-    <row r="43" ht="32" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>75053</v>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>Target is struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
-        <v>23057</v>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 100</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="B42" s="3" t="n">
+        <v>75051</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 16000</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-      <c r="H44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
-        <v>23058</v>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 200</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="B43" s="3" t="n">
+        <v>75052</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 32000</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-      <c r="H45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="n">
-        <v>23059</v>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 300</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-      <c r="H46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="n">
-        <v>23060</v>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 400</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-      <c r="H47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>23061</v>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 500</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-      <c r="H48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>23062</v>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 600</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
-      <c r="H49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="n">
-        <v>23063</v>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 700</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-      <c r="H50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="n">
-        <v>23064</v>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 800</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="n">
-        <v>23065</v>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 900</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="n">
-        <v>23066</v>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="n">
-        <v>75043</v>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-      <c r="H54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>75044</v>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 2000</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-      <c r="H55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="n">
-        <v>75045</v>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 3000</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-      <c r="H56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="n">
-        <v>75046</v>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 4000</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
-      <c r="H57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="n">
-        <v>75047</v>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 5000</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-      <c r="H58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="n">
-        <v>75048</v>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 6000</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-      <c r="H59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="n">
-        <v>75049</v>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 7000</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-      <c r="H60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="n">
-        <v>75050</v>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 8000</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="n">
-        <v>75051</v>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 16000</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr"/>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
-      <c r="H62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="n">
-        <v>75052</v>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 32000</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr"/>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H63"/>
+  <autoFilter ref="A1:H43"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -5076,26 +4478,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add Sucking Wound and update Chronicles of War spell details.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -26,11 +26,11 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$H$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
@@ -2361,7 +2361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2447,180 +2447,276 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Falling Debris</t>
+          <t>Sucking Wound</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>75122</v>
+        <v>75116</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 450000</t>
+          <t>Decrease Current Hit Points by 20000 per Tick</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>1m 12s</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
+          <t>Your open wounds bleed heavily as you move.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Your wounds are no longing bleeding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Sucking Wound</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>75117</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 150000 per Tick</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>1m 12s</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Your open wounds bleed heavily as you move.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Your wounds are no longing bleeding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Sucking Wound</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>75118</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 450500 per Tick</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>1m 12s</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Your open wounds bleed heavily as you move.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Your wounds are no longing bleeding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Falling Debris</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>75122</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 450000</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>Debris, thrown from outside the arena, pummels you.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Black Listed</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B7" s="5" t="n">
         <v>75126</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 500500 per Tick
 Cast on Duration Fade: Black Listed</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Taurlton's gaze rests uneasily on you.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Taurlton's gaze is broken by the falling debris.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Black Listed</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>75127</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600500
 Cast on Fade: Black Listed</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>A shockwave of debris cuts into you.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Black Listed</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>75128</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 4000000000</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Taurlton's gaze shatters your body.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Back of the Line</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B10" s="3" t="n">
         <v>75129</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 75500</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>A shockwave attempts to throw you, but you hold firm.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Back of the Line</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B11" s="3" t="n">
         <v>75130</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 750500
 Fling</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>A shockwave of pressure crushes your bones and throws you.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2629,6 +2725,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>
@@ -3124,7 +3223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3341,79 +3440,111 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>Self-Immolation Effect</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>75010</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 75684 per Tick</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>You have ignited yourself with your self-immolation spell!</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Target has been ignited by a self-immolation spell.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Minotaur Gore</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B8" s="3" t="n">
         <v>75013</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 650000</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Sharpened horns gore your flesh.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Target is gored by sharpened horns.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Decapitating Chop</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>75014</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 4000000000</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>You are slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Target is slain by a mighty cleave.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="64" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="64" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Malaise</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B10" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Decrease Cold Resist by 20
 Decrease Magic Resist by 20
@@ -3421,109 +3552,241 @@
 Decrease Fire Resist by 20</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>14m</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>You feel somewhat vulnerable.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Target looks somewhat uncomfortable.</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>Your vulnerability fades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="64" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Spite</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>40778</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 25000 per Tick (Scales, Base Level: 105)
-Decrease Current Mana by 10000 per Tick (Scales, Base Level: 105) (v417)</t>
-        </is>
-      </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>3 ticks</t>
+          <t>14m</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>You are filled with a sense of bitter spite.</t>
+          <t>You feel somewhat vulnerable.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Target is knocked back.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+          <t>Target looks somewhat uncomfortable.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Your vulnerability fades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Spite of Meldrath</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>75015</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Increase Corruption Counter by 16
+Cast on Duration Fade: Spite of Meldrath Effect</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Corruption 16</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>You feel Meldrath's hatred course through you.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Target shivers as the curse takes hold.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Spite of Meldrath Effect</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>75016</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 650000</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in an explosion of pure spite.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in an explosion of pure spite.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>Stinking Miasma</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B13" s="5" t="n">
         <v>75061</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600000 per Tick
 Decrease Current Mana by 6000 per Tick
 Decrease Current Endurance by 1500 per Tick</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>You are engulfed in the miasma.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Target is caught in the miasma.</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Your lungs clear.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="96" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>75017</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 300000</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>75018</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 600000</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>75019</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 600000</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Spirit Cleaver</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B17" s="5" t="n">
         <v>75024</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Decrease Attack by 500
 Decrease Current Hit Points by 122500 per Tick
@@ -3533,108 +3796,108 @@
 Increase Poison Counter by 297</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Poison 297</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>3m 36s</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>An invisible force of rage splits your soul in two.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Target's soul splits in two.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>You feel whole again.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Soul Consumption</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B18" s="3" t="n">
         <v>75056</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 375000
 Decrease Current Mana by 2700</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Target staggers for a moment.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Spear of Discord</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B19" s="5" t="n">
         <v>75057</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 425000
 Stun NPC for 10s (PC for 5.25s)</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Target is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="96" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Wave of Rage</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B20" s="3" t="n">
         <v>75023</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Increase Spell Mana Cost by 1% to 50%
 Decrease Current Hit Points by 325000
@@ -3644,469 +3907,421 @@
 Increase Poison Counter by 396</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Poison 396</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Target succumbs to the temptation of rage.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
-    </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Ikaav Venom</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B21" s="5" t="n">
         <v>17057</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 7500
 Decrease Current Hit Points by 5000 per Tick
 Increase Poison Counter by 50</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Poison 50</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>10m</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Poison courses through your system after you were bitten.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Target Poison courses through their system after they were bitten.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>You sigh in relief as the poison fades away.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Discord's Rebuke</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B22" s="3" t="n">
         <v>75025</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 475000</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Chaos fills your mind and pains your soul.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Target jerks and spasms in pain.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Vis Percussio</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
-        <v>48039</v>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="B23" s="5" t="n">
+        <v>75033</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Vis Percussio</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>75033</v>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Vita Anuimis</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>75034</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>48040</v>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Vita Anuimis</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>75034</v>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B25" s="5" t="n">
         <v>75031</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 222000 per Tick
 Decrease Melee Haste by 55%</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B26" s="5" t="n">
         <v>75039</v>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Decrease Melee Haste by 55% (v371, Incremental)
 Decrease Current Hit Points by 150000 per Tick</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
+      <c r="B27" s="3" t="n">
         <v>75030</v>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 325000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr"/>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B28" s="3" t="n">
         <v>75035</v>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Claustro Facultis</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B29" s="5" t="n">
         <v>75036</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 275000
 Decrease Current Mana by 3510 (v417)</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Magic drains painfully from your body.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Repenta Vitoris</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B30" s="3" t="n">
         <v>75032</v>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 456789 per Tick</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>A ball of electricity gathers around you.</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Ignas Maxio</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B31" s="5" t="n">
         <v>75037</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 299000 per Tick
 Decrease Movement Speed by 65%</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Flames engulf you.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Humas Maxio</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B32" s="3" t="n">
         <v>75038</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 444000
 Push Back 3 Units and Up 3 Units
 Stun for 2s</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>You are engulfed in grinding earth.</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Gravitas Maxio</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B33" s="5" t="n">
         <v>75040</v>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
 Decrease Current Hit Points by 175000 per Tick</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>You feel the very earth pulling you apart.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="64" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="64" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Resonating Beam</t>
         </is>
       </c>
-      <c r="B31" s="5" t="n">
+      <c r="B34" s="3" t="n">
         <v>75058</v>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Dispel Beneficial (100% Chance)
 Decrease Current Hit Points by 600000
@@ -4114,327 +4329,327 @@
 Decrease Current Endurance by 1850</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>You are hit by a powerful resonation.</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Repulsion of the First Creation</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B35" s="5" t="n">
         <v>75042</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 125000
 Push Back 3 Units and Up 12 Units</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>You are repulsed.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>Target is repulsed.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Retribution of the First Creation</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
+      <c r="B36" s="3" t="n">
         <v>75053</v>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 325000</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Target is struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="n">
-        <v>75043</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="n">
-        <v>75044</v>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 2000</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="n">
-        <v>75045</v>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 3000</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr">
         <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Target is struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>75043</v>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 1000</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B38" s="5" t="n">
+        <v>75044</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 2000</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr"/>
+      <c r="H38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>75045</v>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 3000</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
         <v>75046</v>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 4000</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="F40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr"/>
+      <c r="H40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B41" s="5" t="n">
         <v>75047</v>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 5000</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-      <c r="H38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B42" s="5" t="n">
         <v>75048</v>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 6000</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-      <c r="H39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B43" s="5" t="n">
         <v>75049</v>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 7000</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B44" s="5" t="n">
         <v>75050</v>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 8000</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B45" s="5" t="n">
         <v>75051</v>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 16000</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-      <c r="H42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>Lava Elemental Protection</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B46" s="5" t="n">
         <v>75052</v>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Increase Damage Shield by 32000</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>5d</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr"/>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -4478,6 +4693,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Keep placeholder and writeup spell rules in the site scripts.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -3535,7 +3535,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr"/>
     </row>
-    <row r="10" ht="64" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Malaise</t>
@@ -3546,10 +3546,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Decrease Cold Resist by 20
-Decrease Magic Resist by 20
-Decrease Poison Resist by 20
-Decrease Fire Resist by 20</t>
+          <t>Place Holder</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Barb Shot to the Moruuk and Sorshkah writeup.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$H$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
@@ -1964,7 +1964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2059,251 +2059,284 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>Barb Shot</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>75133</v>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 650000
+Stun for 20s</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Sharp barbs dig deep into you draining your strength.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>The barbs fall loose, allowing you to recover.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B4" s="3" t="n">
         <v>75134</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B5" s="3" t="n">
         <v>75135</v>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B6" s="3" t="n">
         <v>75151</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Fling</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B7" s="3" t="n">
         <v>75152</v>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Fling</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Lockjaw Trap</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>75137</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Root</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>The razor sharp jaws of the trap cut into your leg.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>Your wounds close.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Slow Your Roll</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B9" s="3" t="n">
         <v>75138</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 750000
 Decrease Melee Haste by 10% (v371, Incremental)
 Increase Cast Time by 1s</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Moruuk's blow rattles you, slowing your reactions.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>You shake off the attack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Stronger Together</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>75141</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Increase Melee Haste by 25%</t>
-        </is>
-      </c>
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Moruuk's blow rattles you, slowing your reactions.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>You shake off the attack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Stronger Together</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>75141</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Increase Melee Haste by 25%</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Target's attacks become faster and more aggressive.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Taking Your Stuff</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B11" s="3" t="n">
         <v>75140</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Mana by 0.1% of Total Mana, Max: 0
 Decrease Current Endurance by 0.1% of Total Endurance, Max: 0</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>You feel drained.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="80" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Aura of Greed</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B12" s="5" t="n">
         <v>75147</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2311,30 +2344,30 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>The weight of your poverty takes its toll.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Aura of Poverty</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="3" t="n">
         <v>75148</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2342,22 +2375,22 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>The weight of your greed takes its toll.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12"/>
+  <autoFilter ref="A1:H13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2370,6 +2403,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add Creeping Madness stacks to Fractured Vazaelle.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
@@ -2811,7 +2811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2909,350 +2909,511 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Fractured Psyche</t>
+          <t>Creeping Madness</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>75100</v>
+        <v>75095</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 800800</t>
+          <t>Decrease Current Hit Points by 1000 per Tick</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Instant</t>
+          <t>2m</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Your mind fractures and all you feel is agony.</t>
+          <t>The maddening influence of the realm seeps in.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Silencing Mist</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>75101</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Inhibit Spell Casting (Spell Silence)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>2 ticks</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>The mist clings to your throat, preventing you from speaking.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>The mist clears, you can speak again.</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Creeping Madness</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>75096</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1000 per Tick</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>The maddening influence of the realm tickles your mind.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Creeping Madness</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>75097</v>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1000 per Tick</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>The maddening influence of the realm clouds your senses.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Creeping Madness</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>75098</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1000 per Tick</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>2m</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>The maddening influence of the realm whispers in your ear.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Creeping Madness</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>75099</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 1000 per Tick
+Charm up to Level 300</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>The maddening influence of the realm overwhelms you.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Fractured Psyche</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>75100</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 800800</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Your mind fractures and all you feel is agony.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Silencing Mist</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>75101</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Inhibit Spell Casting (Spell Silence)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>The mist clings to your throat, preventing you from speaking.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>The mist clears, you can speak again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Psychic Shriek</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B10" s="3" t="n">
         <v>75103</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600500 per Tick
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>A piercing shriek rattles your mind.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Your mind clears</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Psychic Blast</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B11" s="5" t="n">
         <v>75104</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 800800</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Psychic energy rends your mind.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Psychic Blast</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B12" s="5" t="n">
         <v>75105</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Cap Hit Points at 25%</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>Psychic energy shatters your spirit.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>You pull yourself together.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B13" s="3" t="n">
         <v>75107</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 250000
 Fling</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>You have been judged and found wanting.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B14" s="3" t="n">
         <v>75108</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Decrease Armor Class by 994 to 1313, Based on Class</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Vazaelle's judgement makes it difficult to defend yourself.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>You can defend yourself again.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B15" s="3" t="n">
         <v>75109</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 650000
 Fling
 Decrease Armor Class by 994 to 1313, Based on Class</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>You have been judged and found wanting.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Tainted Affliction</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B16" s="5" t="n">
         <v>75110</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 450000 per Tick</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Corrupting influence breaks your mind and body.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>The corrupting influence fades.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Arcing Slash</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B17" s="3" t="n">
         <v>75111</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 700750 per Tick</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>A quick slash causes you to bleed.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>The bleeding stops.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Wither</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B18" s="5" t="n">
         <v>75113</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000 per Tick
 Increase Corruption Counter by 30</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Corruption 30</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Corruption drains your life essence.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>The corruption dissipates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H18"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3266,6 +3427,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add Queasy and Sickening Glob to the Moruuk and Sorshkah writeup.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Dipuc'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scorn'!$A$1:$H$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Scorn'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Moruuk and Sorshkah'!$A$1:$H$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
@@ -1964,7 +1964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2019,324 +2019,391 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Queasy</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>75131</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Increase Poison Counter by 60</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Poison 60</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Sorshkah has shaken off the sickness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
           <t>Feral Toxin</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B3" s="5" t="n">
         <v>75132</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Increase Poison Counter by 120
 Decrease Current Hit Points by 550000 per Tick</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Poison 120</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>You inhale a potent toxin that burns your lungs.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>The poison runs its course.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Barb Shot</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B4" s="3" t="n">
         <v>75133</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 650000
 Stun for 20s</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Sharp barbs dig deep into you draining your strength.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>The barbs fall loose, allowing you to recover.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B5" s="5" t="n">
         <v>75134</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B6" s="5" t="n">
         <v>75135</v>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>The manticore's claws rake across your flesh.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B7" s="5" t="n">
         <v>75151</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Fling</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Rake</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B8" s="5" t="n">
         <v>75152</v>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Fling</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>The manticore's claws strike throws you back.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sickening Glob</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>75136</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 500000 per Tick
+Decrease Movement Speed by 25%
+Decrease Melee Haste by 10% (v371, Incremental)
+Increase Cast Time by 1s</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>3 ticks</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Putrid phlegm burns your skin and invades your senses.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Fresh air, finally!</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Lockjaw Trap</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B10" s="5" t="n">
         <v>75137</v>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600600
 Root</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>The razor sharp jaws of the trap cut into your leg.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Your wounds close.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Slow Your Roll</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B11" s="3" t="n">
         <v>75138</v>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 750000
 Decrease Melee Haste by 10% (v371, Incremental)
 Increase Cast Time by 1s</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Moruuk's blow rattles you, slowing your reactions.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>You shake off the attack.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Stronger Together</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B12" s="5" t="n">
         <v>75141</v>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Increase Melee Haste by 25%</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>Target's attacks become faster and more aggressive.</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Taking Your Stuff</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B13" s="3" t="n">
         <v>75140</v>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Mana by 0.1% of Total Mana, Max: 0
 Decrease Current Endurance by 0.1% of Total Endurance, Max: 0</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>You feel drained.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="80" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Aura of Greed</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B14" s="5" t="n">
         <v>75147</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2344,30 +2411,30 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>The weight of your poverty takes its toll.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="80" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Aura of Poverty</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B15" s="3" t="n">
         <v>75148</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Decrease Hit Damage by 50% (v185)
 Decrease Spell Damage by 1% to 50% (v124, Before DoT Crit, After DD Crit)
@@ -2375,22 +2442,22 @@
 Increase Spell Damage Taken by 50% (v296, Before Crit)</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>20m</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>The weight of your greed takes its toll.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H13"/>
+  <autoFilter ref="A1:H15"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -2404,6 +2471,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Add Grasping Mist to the Fractured Vazaelle writeup.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Moruuk and Sorshkah'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Taurlton'!$A$1:$H$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
@@ -2880,7 +2880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3199,290 +3199,323 @@
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Grasping Mist</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>75102</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Root
+Increase Chance of Root Breaking by 0%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>The mist grips your feet, holding you in place.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>The mist clears, you can move again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Psychic Shriek</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B11" s="5" t="n">
         <v>75103</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600500 per Tick
 Inhibit Spell Casting (Spell Silence)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>4 ticks</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>A piercing shriek rattles your mind.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Your mind clears</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Psychic Blast</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>75104</v>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 800800</t>
-        </is>
-      </c>
       <c r="D11" s="4" t="inlineStr"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
+          <t>4 ticks</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>A piercing shriek rattles your mind.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Your mind clears</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Psychic Blast</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>75104</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 800800</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Psychic energy rends your mind.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Psychic Blast</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B13" s="3" t="n">
         <v>75105</v>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Cap Hit Points at 25%</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Psychic energy shatters your spirit.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>You pull yourself together.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B14" s="5" t="n">
         <v>75107</v>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 250000
 Fling</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="4" t="inlineStr">
         <is>
           <t>You have been judged and found wanting.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr"/>
-      <c r="H13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B15" s="5" t="n">
         <v>75108</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Decrease Armor Class by 994 to 1313, Based on Class</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>60s</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Vazaelle's judgement makes it difficult to defend yourself.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>You can defend yourself again.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Dread Judgement</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B16" s="5" t="n">
         <v>75109</v>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 650000
 Fling
 Decrease Armor Class by 994 to 1313, Based on Class</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>You have been judged and found wanting.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Tainted Affliction</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>75110</v>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 450000 per Tick</t>
-        </is>
-      </c>
       <c r="D16" s="4" t="inlineStr"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>5 ticks</t>
+          <t>Instant</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Corrupting influence breaks your mind and body.</t>
+          <t>You have been judged and found wanting.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>The corrupting influence fades.</t>
-        </is>
-      </c>
+      <c r="H16" s="4" t="inlineStr"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Arcing Slash</t>
+          <t>Tainted Affliction</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>75111</v>
+        <v>75110</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Decrease Current Hit Points by 700750 per Tick</t>
+          <t>Decrease Current Hit Points by 450000 per Tick</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>60s</t>
+          <t>5 ticks</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>A quick slash causes you to bleed.</t>
+          <t>Corrupting influence breaks your mind and body.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
+          <t>The corrupting influence fades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Arcing Slash</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>75111</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 700750 per Tick</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>60s</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>A quick slash causes you to bleed.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
           <t>The bleeding stops.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Wither</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B19" s="3" t="n">
         <v>75113</v>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000 per Tick
 Increase Corruption Counter by 30</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Corruption 30</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Corruption drains your life essence.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>The corruption dissipates</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -3501,6 +3534,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Restore Chronicles spell links the audit replaced with forum typos.
</commit_message>
<xml_diff>
--- a/Info/FoF_Raid_Spells.xlsx
+++ b/Info/FoF_Raid_Spells.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Taurlton'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Fractured Vazaelle'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Fractured Vazaelle'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Chronicles of War'!$A$1:$H$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Chronicles of War'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Eriak Zek'!$A$1:$H$30</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Eriak Zek'!$1:$1</definedName>
@@ -3555,7 +3555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3772,153 +3772,350 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>Self-Immolation Effect</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>75010</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 75684 per Tick</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>2 ticks</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>You have ignited yourself with your self-immolation spell!</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Target has been ignited by a self-immolation spell.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Minotaur Gore</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B8" s="3" t="n">
         <v>75013</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 650000</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Sharpened horns gore your flesh.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Target is gored by sharpened horns.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Decapitating Chop</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B9" s="5" t="n">
         <v>75014</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Feign Death (1% Chance)
 Decrease Current Hit Points by 4000000000</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>You are slain by a mighty cleave.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Target is slain by a mighty cleave.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Malaise</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Place Holder</t>
-        </is>
-      </c>
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>You are slain by a mighty cleave.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Target is slain by a mighty cleave.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Malaise</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Place Holder</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>14m</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>You feel somewhat vulnerable.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Target looks somewhat uncomfortable.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Your vulnerability fades.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Spite of Meldrath</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>75015</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Increase Corruption Counter by 16
+Cast on Duration Fade: Spite of Meldrath Effect</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Corruption 16</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>5 ticks</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>You feel Meldrath's hatred course through you.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Target shivers as the curse takes hold.</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Spite of Meldrath Effect</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>75016</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 650000</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in an explosion of pure spite.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in an explosion of pure spite.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Stinking Miasma</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B13" s="5" t="n">
         <v>75061</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 600000 per Tick
 Decrease Current Mana by 6000 per Tick
 Decrease Current Endurance by 1500 per Tick</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>You are engulfed in the miasma.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Target is caught in the miasma.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>Your lungs clear.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="96" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>75017</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 300000</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>75018</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 600000</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Tick-Tock Explosion</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>75019</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 600000</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>You are caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Target is caught in the explosion.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Spirit Cleaver</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B17" s="5" t="n">
         <v>75024</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Decrease Attack by 500
 Decrease Current Hit Points by 122500 per Tick
@@ -3928,108 +4125,108 @@
 Increase Poison Counter by 297</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Poison 297</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>3m 36s</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>An invisible force of rage splits your soul in two.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>Target's soul splits in two.</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>You feel whole again.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Soul Consumption</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B18" s="3" t="n">
         <v>75056</v>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 375000
 Decrease Current Mana by 2700</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>An invisible force tugs at your soul.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Target staggers for a moment.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Spear of Discord</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B19" s="5" t="n">
         <v>75057</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 425000
 Stun NPC for 10s (PC for 5.25s)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Your body is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>Target is pierced by the spear of discord.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
-    </row>
-    <row r="14" ht="96" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Wave of Rage</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B20" s="3" t="n">
         <v>75023</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Increase Spell Mana Cost by 1% to 50%
 Decrease Current Hit Points by 325000
@@ -4039,421 +4236,421 @@
 Increase Poison Counter by 396</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Poison 396</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Your spirit is overcome by a wave of rage.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Target succumbs to the temptation of rage.</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Ikaav Venom</t>
         </is>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B21" s="5" t="n">
         <v>17057</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 7500
 Decrease Current Hit Points by 5000 per Tick
 Increase Poison Counter by 50</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Poison 50</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>10m</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Poison courses through your system after you were bitten.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Target Poison courses through their system after they were bitten.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>You sigh in relief as the poison fades away.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Discord's Rebuke</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B22" s="3" t="n">
         <v>75025</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 475000</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Chaos fills your mind and pains your soul.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Target jerks and spasms in pain.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Vis Percussio</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B23" s="5" t="n">
         <v>75033</v>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Cast on Skill Use: Vis Percussio Proc (5)</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr"/>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>Vita Anuimis</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B24" s="3" t="n">
         <v>75034</v>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Cast on Skill Use: Vita Anuimis Proc (5)</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>4 ticks</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
-      <c r="H18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B25" s="5" t="n">
         <v>75031</v>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 222000 per Tick
 Decrease Melee Haste by 55%</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr"/>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Vita Tardius</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>75039</v>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Decrease Melee Haste by 55% (v371, Incremental)
 Decrease Current Hit Points by 150000 per Tick</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>5 ticks</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Your body convulses as electricity runs through you.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr"/>
+      <c r="H26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B27" s="3" t="n">
         <v>75030</v>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 325000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Claustro Vitoris</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B28" s="3" t="n">
         <v>75035</v>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 350000
 Stun for 1s</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>You are shocked!</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>Claustro Facultis</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
+      <c r="B29" s="5" t="n">
         <v>75036</v>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 275000
 Decrease Current Mana by 3510 (v417)</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Magic drains painfully from your body.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Repenta Vitoris</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B30" s="3" t="n">
         <v>75032</v>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 456789 per Tick</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>A ball of electricity gathers around you.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Ignas Maxio</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B31" s="5" t="n">
         <v>75037</v>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 299000 per Tick
 Decrease Movement Speed by 65%</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>3 ticks</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Flames engulf you.</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Humas Maxio</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B32" s="3" t="n">
         <v>75038</v>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 444000
 Push Back 3 Units and Up 3 Units
 Stun for 2s</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>You are engulfed in grinding earth.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Gravitas Maxio</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B33" s="5" t="n">
         <v>75040</v>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Gradual Pull to 0 Units Away (Force=110) up to Your Level
 Decrease Current Hit Points by 175000 per Tick</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>2 ticks</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>You feel the very earth pulling you apart.</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28" ht="64" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="64" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Resonating Beam</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B34" s="3" t="n">
         <v>75058</v>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Dispel Beneficial (100% Chance)
 Decrease Current Hit Points by 600000
@@ -4461,228 +4658,84 @@
 Decrease Current Endurance by 1850</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Instant</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>You are hit by a powerful resonation.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr"/>
-      <c r="H28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="32" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Repulsion of the First Creation</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
+      <c r="B35" s="5" t="n">
         <v>75042</v>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Decrease Current Hit Points by 125000
 Push Back 3 Units and Up 12 Units</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>You are repulsed.</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Target is repulsed.</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Retribution of the First Creation</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="n">
-        <v>75053</v>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>Decrease Current Hit Points by 325000</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>Instant</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>You are struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Target is struck by the retribution of The First Creation.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>75043</v>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 1000</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>75044</v>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 2000</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
-      <c r="G32" s="4" t="inlineStr"/>
-      <c r="H32" s="4" t="inlineStr"/>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>75045</v>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 3000</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr"/>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
-      <c r="G33" s="4" t="inlineStr"/>
-      <c r="H33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="n">
-        <v>75046</v>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 4000</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr"/>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr"/>
-      <c r="G34" s="4" t="inlineStr"/>
-      <c r="H34" s="4" t="inlineStr"/>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>75047</v>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 5000</t>
-        </is>
-      </c>
       <c r="D35" s="4" t="inlineStr"/>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr"/>
-      <c r="G35" s="4" t="inlineStr"/>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>You are repulsed.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Target is repulsed.</t>
+        </is>
+      </c>
       <c r="H35" s="4" t="inlineStr"/>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>Lava Elemental Protection</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>75048</v>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Increase Damage Shield by 6000</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr"/>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="4" t="inlineStr"/>
-      <c r="H36" s="4" t="inlineStr"/>
+    <row r="36" ht="32" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Retribution of the First Creation</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>75053</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Decrease Current Hit Points by 325000</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Instant</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>You are struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Target is struck by the retribution of The First Creation.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
@@ -4691,11 +4744,11 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>75049</v>
+        <v>75043</v>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 7000</t>
+          <t>Increase Damage Shield by 1000</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr"/>
@@ -4715,11 +4768,11 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>75050</v>
+        <v>75044</v>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 8000</t>
+          <t>Increase Damage Shield by 2000</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr"/>
@@ -4739,11 +4792,11 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>75051</v>
+        <v>75045</v>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 16000</t>
+          <t>Increase Damage Shield by 3000</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr"/>
@@ -4763,11 +4816,11 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>75052</v>
+        <v>75046</v>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Increase Damage Shield by 32000</t>
+          <t>Increase Damage Shield by 4000</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr"/>
@@ -4780,8 +4833,152 @@
       <c r="G40" s="4" t="inlineStr"/>
       <c r="H40" s="4" t="inlineStr"/>
     </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>75047</v>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 5000</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>75048</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 6000</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr"/>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr"/>
+      <c r="H42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>75049</v>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 7000</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>75050</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 8000</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>75051</v>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 16000</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr"/>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Lava Elemental Protection</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>75052</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Increase Damage Shield by 32000</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr"/>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>5d</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H40"/>
+  <autoFilter ref="A1:H46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
@@ -4822,6 +5019,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="3" fitToHeight="0" fitToWidth="1"/>

</xml_diff>